<commit_message>
final upload + docker and deployment guide
</commit_message>
<xml_diff>
--- a/rag-data/providers/Fatima/excel/metadata.xlsx
+++ b/rag-data/providers/Fatima/excel/metadata.xlsx
@@ -473,27 +473,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>AI Development Services – Fatima Fatima is a professional AI developer providing end-to-end AI
-solutions, including chatbots, automation apps, predictive analytics systems, and custom machine
-learning tools. Services Offered Custom Chatbot Development (RAG, LLM-Based) AI Automation
-Integrations (API-based, workflow automation) Predictive Analytics &amp; Data Modeling Fine-tuning and
-Prompt Engineering AI-powered dashboard integrations Consultation on AI architecture and
-deployment Timings &amp; Availability Fatima is available Monday to Saturday from 10 AM – 7 PM
-(GMT+5). Urgent consultations may be scheduled outside regular hours upon request. Charges Initial
-Frequently Asked Questions (FAQ) 1. How long does it take to develop an AI chatbot? Typical
-development time is 3–7 days depending on requirements such as integrations, UI, and model
-configuration. 2. Do you provide deployment services? Yes. Deployment is offered for web apps, cloud
-environments, and messaging platforms (WhatsApp, Telegram, etc.). 3. What do you need from the
-client? Project requirements Sample data (optional) Preferred platform or integration method Budget
-and timeline expectations 4. Is data kept confidential? Yes. Data confidentiality is ensured, and NDAs
-can be signed if required. 5. Do you offer ongoing support? Yes. Monthly support plans are available
-and can be customized. Contact Information Name: Fatima
-Email: fatima.ai.services@example.com</t>
+          <t>Test services: alpha, beta, gamma</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>See provider pricing</t>
+          <t>Variable</t>
         </is>
       </c>
     </row>

</xml_diff>